<commit_message>
fix(km19): số phiến dầm Super-T theo chủ dự án: 2 S1B1 + 3 S1B2 + 1 S1B3 + 9 S1G
- Chủ dự án soát 11/10/2026. Khớp sơ đồ bố trí nhịp tr.75 (chú giải có S1B3 — OCR đọc nhầm một ký hiệu
  S1B3 thành S1B1 nên trước đây suy ra 3 S1B1).
- Hồ sơ OCR không có bảng thép riêng cho S1B3 (tr.86–94 chỉ có S1B1, S1B2, S1G): tạm dùng bảng S1B1 tr.88,
  đánh dấu NGHI VẤN. Tổng 89.690,31 kg vẫn khớp tr.175 (77,743 + 11,947 t) — chỉ khớp khi S1B3 = S1B1.
- BBS tách dòng S1B3 riêng; dự toán F67 = 2×S1B1 + 3×S1B2 + S1B3 + 9×S1G. Tổng tiền không đổi.
- Bộ file cắt thép sinh lại ở commit sau.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/08_Du_Toan_GXD_Thong_Tu_11_2021.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/08_Du_Toan_GXD_Thong_Tu_11_2021.xlsx
@@ -3540,7 +3540,7 @@
       <c r="B67" s="21" t="n"/>
       <c r="C67" s="22" t="inlineStr">
         <is>
-          <t>- Cốt thép thường 15 phiến: 3 × S1B1 (tr.88) + 3 × S1B2 (tr.91) + 9 × S1G (tr.94)</t>
+          <t>- Cốt thép thường 15 phiến: 2 × S1B1 (tr.88) + 3 × S1B2 (tr.91) + 1 × S1B3 (bảng S1B1 tr.88) + 9 × S1G (tr.94)</t>
         </is>
       </c>
       <c r="D67" s="23" t="inlineStr">
@@ -3552,7 +3552,7 @@
         <v>1</v>
       </c>
       <c r="F67" s="35">
-        <f>3*6.07125+3*6.06528+9*5.92008</f>
+        <f>2*6.07125+3*6.06528+6.07125+9*5.92008</f>
         <v/>
       </c>
       <c r="G67" s="35" t="n">
@@ -3572,7 +3572,7 @@
       <c r="L67" s="21" t="n"/>
       <c r="M67" s="38" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 90,630 → 89,690. Dòng tiêu đề cũ ghi cứng 361,596 t (= BBS cũ, gấp khoảng 4 lần bản vẽ). Bản vẽ: 89,690 t = tr.175 (77,743 + 11,947 t). Số phiến 3/3/9 suy từ tổng tr.175 — xác nhận theo mặt cắt ngang.</t>
+          <t>Theo bản vẽ: 90,630 → 89,690. Dòng tiêu đề cũ ghi cứng 361,596 t (= BBS cũ, gấp khoảng 4 lần bản vẽ). Số phiến 2/3/1/9 theo chủ dự án (sơ đồ tr.75). Hồ sơ không có bảng thép S1B3 — tạm dùng bảng S1B1; tổng 89,690 t khớp tr.175 (77,743 + 11,947 t).</t>
         </is>
       </c>
       <c r="N67" t="n">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="E37" s="42" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 90,630 → 89,690. Dòng tiêu đề cũ ghi cứng 361,596 t (= BBS cũ, gấp khoảng 4 lần bản vẽ). Bản vẽ: 89,690 t = tr.175 (77,743 + 11,947 t). Số phiến 3/3/9 suy từ tổng tr.175 — xác nhận theo mặt cắt ngang.</t>
+          <t>Theo bản vẽ: 90,630 → 89,690. Dòng tiêu đề cũ ghi cứng 361,596 t (= BBS cũ, gấp khoảng 4 lần bản vẽ). Số phiến 2/3/1/9 theo chủ dự án (sơ đồ tr.75). Hồ sơ không có bảng thép S1B3 — tạm dùng bảng S1B1; tổng 89,690 t khớp tr.175 (77,743 + 11,947 t).</t>
         </is>
       </c>
       <c r="F37" s="42" t="inlineStr">

</xml_diff>

<commit_message>
fix(km19): giữ hệ số nở thành 1,12 cho bê tông cọc khoan nhồi (quyết định chủ dự án)
- Dự toán dòng QS 18–21: thể tích thiết kế từng cọc (tr.64/66/68/70, gồm bê tông đầu cọc) × số cọc ×
  hệ số nở thành 1,12 (cột I). Bê tông cọc 1.006,54 → 1.127,33 m³ (dự toán cũ 1.104,56 m³ tính
  π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc).
- tools/estimate_reconcile.py: dòng sửa nhận hệ số I từ cấu hình (mặc định 1).
- G_XD 26,78 → 27,03 tỷ (27.029.878.097 đ); 03a đề nghị kỳ này 10,61 tỷ (tỷ lệ hoàn thành vẫn NGHI VẤN).
- Tính lại bằng LibreOffice: 0 lỗi công thức.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/08_Du_Toan_GXD_Thong_Tu_11_2021.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/03_KINH_TE_QS_DU_TOAN_THANH_TOAN/08_Du_Toan_GXD_Thong_Tu_11_2021.xlsx
@@ -1560,7 +1560,7 @@
       <c r="B18" s="21" t="n"/>
       <c r="C18" s="22" t="inlineStr">
         <is>
-          <t>- Bê tông 3 cọc mố M1 L=20m (bản vẽ tr.64, gồm bê tông đầu cọc)</t>
+          <t>- Bê tông 3 cọc mố M1 L=20m (bản vẽ tr.64, gồm bê tông đầu cọc) × hệ số nở thành 1,12</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
@@ -1581,7 +1581,7 @@
         <v>1</v>
       </c>
       <c r="I18" s="36" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="J18" s="37">
         <f>E18*F18*G18*H18*I18</f>
@@ -1591,7 +1591,7 @@
       <c r="L18" s="21" t="n"/>
       <c r="M18" s="38" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 76,002 → 70,740. Bỏ hệ số I = 3,5186 (π × 1,12 nở thành): lấy thể tích thiết kế tr.64. Nếu hợp đồng cho tính nở thành thì ghim lại hệ số.</t>
+          <t>Theo bản vẽ: 76,002 → 79,229. Thể tích thiết kế tr.64 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="N18" t="n">
@@ -1603,7 +1603,7 @@
       <c r="B19" s="21" t="n"/>
       <c r="C19" s="22" t="inlineStr">
         <is>
-          <t>- Bê tông 8 cọc trụ T1 L=40m (bản vẽ tr.68, gồm bê tông đầu cọc)</t>
+          <t>- Bê tông 8 cọc trụ T1 L=40m (bản vẽ tr.68, gồm bê tông đầu cọc) × hệ số nở thành 1,12</t>
         </is>
       </c>
       <c r="D19" s="23" t="inlineStr">
@@ -1624,7 +1624,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="36" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="J19" s="37">
         <f>E19*F19*G19*H19*I19</f>
@@ -1634,7 +1634,7 @@
       <c r="L19" s="21" t="n"/>
       <c r="M19" s="38" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 405,343 → 367,040. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.68.</t>
+          <t>Theo bản vẽ: 405,343 → 411,085. Thể tích thiết kế tr.68 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="N19" t="n">
@@ -1646,7 +1646,7 @@
       <c r="B20" s="21" t="n"/>
       <c r="C20" s="22" t="inlineStr">
         <is>
-          <t>- Bê tông 8 cọc trụ T2 L=30m (bản vẽ tr.70, gồm bê tông đầu cọc)</t>
+          <t>- Bê tông 8 cọc trụ T2 L=30m (bản vẽ tr.70, gồm bê tông đầu cọc) × hệ số nở thành 1,12</t>
         </is>
       </c>
       <c r="D20" s="23" t="inlineStr">
@@ -1667,7 +1667,7 @@
         <v>1</v>
       </c>
       <c r="I20" s="36" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="J20" s="37">
         <f>E20*F20*G20*H20*I20</f>
@@ -1677,7 +1677,7 @@
       <c r="L20" s="21" t="n"/>
       <c r="M20" s="38" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 304,007 → 277,840. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.70.</t>
+          <t>Theo bản vẽ: 304,007 → 311,181. Thể tích thiết kế tr.70 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="N20" t="n">
@@ -1689,7 +1689,7 @@
       <c r="B21" s="21" t="n"/>
       <c r="C21" s="22" t="inlineStr">
         <is>
-          <t>- Bê tông 7 cọc mố M2 L=36m (bản vẽ tr.66, gồm bê tông đầu cọc)</t>
+          <t>- Bê tông 7 cọc mố M2 L=36m (bản vẽ tr.66, gồm bê tông đầu cọc) × hệ số nở thành 1,12</t>
         </is>
       </c>
       <c r="D21" s="23" t="inlineStr">
@@ -1710,7 +1710,7 @@
         <v>1</v>
       </c>
       <c r="I21" s="36" t="n">
-        <v>1</v>
+        <v>1.12</v>
       </c>
       <c r="J21" s="37">
         <f>E21*F21*G21*H21*I21</f>
@@ -1720,7 +1720,7 @@
       <c r="L21" s="21" t="n"/>
       <c r="M21" s="38" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 319,207 → 290,920. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.66.</t>
+          <t>Theo bản vẽ: 319,207 → 325,830. Thể tích thiết kế tr.66 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="N21" t="n">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="E8" s="42" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 76,002 → 70,740. Bỏ hệ số I = 3,5186 (π × 1,12 nở thành): lấy thể tích thiết kế tr.64. Nếu hợp đồng cho tính nở thành thì ghim lại hệ số.</t>
+          <t>Theo bản vẽ: 76,002 → 79,229. Thể tích thiết kế tr.64 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="F8" s="42" t="inlineStr">
@@ -5088,7 +5088,7 @@
       </c>
       <c r="G8" s="42" t="inlineStr">
         <is>
-          <t>70,740</t>
+          <t>79,229</t>
         </is>
       </c>
       <c r="H8" s="42" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="E9" s="42" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 405,343 → 367,040. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.68.</t>
+          <t>Theo bản vẽ: 405,343 → 411,085. Thể tích thiết kế tr.68 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="F9" s="42" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="G9" s="42" t="inlineStr">
         <is>
-          <t>367,040</t>
+          <t>411,085</t>
         </is>
       </c>
       <c r="H9" s="42" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="E10" s="42" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 304,007 → 277,840. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.70.</t>
+          <t>Theo bản vẽ: 304,007 → 311,181. Thể tích thiết kế tr.70 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="F10" s="42" t="inlineStr">
@@ -5166,7 +5166,7 @@
       </c>
       <c r="G10" s="42" t="inlineStr">
         <is>
-          <t>277,840</t>
+          <t>311,181</t>
         </is>
       </c>
       <c r="H10" s="42" t="inlineStr">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="E11" s="42" t="inlineStr">
         <is>
-          <t>Theo bản vẽ: 319,207 → 290,920. Bỏ hệ số nở thành 3,5186 — lấy thể tích thiết kế tr.66.</t>
+          <t>Theo bản vẽ: 319,207 → 325,830. Thể tích thiết kế tr.66 × hệ số nở thành 1,12 (Chủ dự án quyết định 11/10/2026 giữ hệ số nở thành 1,12 cho bê tông cọc). Dự toán cũ: π × 0,6² × L × 1,12, chưa gồm bê tông đầu cọc.</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="G11" s="42" t="inlineStr">
         <is>
-          <t>290,920</t>
+          <t>325,830</t>
         </is>
       </c>
       <c r="H11" s="42" t="inlineStr">

</xml_diff>